<commit_message>
added two new VOs
</commit_message>
<xml_diff>
--- a/lesson_vo_manifest.xlsx
+++ b/lesson_vo_manifest.xlsx
@@ -2796,7 +2796,7 @@
       </c>
       <c r="F49" s="15" t="inlineStr">
         <is>
-          <t>अब दहाइयाँ घटाइए। 4 दहाई में से 2 दहाई हटाइए।</t>
+          <t>अब दहाई घटाइए। 4 दहाई में से 2 दहाई हटाइए।</t>
         </is>
       </c>
       <c r="G49" s="14" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="I49" s="14" t="inlineStr"/>
       <c r="J49" s="12" t="n">
-        <v>5.67</v>
+        <v>5.09</v>
       </c>
       <c r="K49" s="13" t="inlineStr">
         <is>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="F62" s="19" t="inlineStr">
         <is>
-          <t>अब दहाइयाँ घटाइए। 5 दहाई में से 3 दहाई हटाइए।</t>
+          <t>अब दहाई घटाइए। 5 दहाई में से 3 दहाई हटाइए।</t>
         </is>
       </c>
       <c r="G62" s="18" t="inlineStr">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="I62" s="18" t="inlineStr"/>
       <c r="J62" s="16" t="n">
-        <v>5.34</v>
+        <v>5.25</v>
       </c>
       <c r="K62" s="17" t="inlineStr">
         <is>
@@ -7488,7 +7488,7 @@
       </c>
       <c r="D46" s="26" t="inlineStr">
         <is>
-          <t>अब दहाइयाँ घटाइए। 4 दहाई में से 2 दहाई हटाइए।</t>
+          <t>अब दहाई घटाइए। 4 दहाई में से 2 दहाई हटाइए।</t>
         </is>
       </c>
       <c r="E46" s="27" t="inlineStr">
@@ -7497,7 +7497,7 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>5.67</v>
+        <v>5.09</v>
       </c>
       <c r="G46" s="25" t="inlineStr">
         <is>
@@ -7785,7 +7785,7 @@
       </c>
       <c r="D55" s="26" t="inlineStr">
         <is>
-          <t>अब दहाइयाँ घटाइए। 5 दहाई में से 3 दहाई हटाइए।</t>
+          <t>अब दहाई घटाइए। 5 दहाई में से 3 दहाई हटाइए।</t>
         </is>
       </c>
       <c r="E55" s="27" t="inlineStr">
@@ -7794,7 +7794,7 @@
         </is>
       </c>
       <c r="F55" s="24" t="n">
-        <v>5.34</v>
+        <v>5.25</v>
       </c>
       <c r="G55" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
removed shabash word from VO
</commit_message>
<xml_diff>
--- a/lesson_vo_manifest.xlsx
+++ b/lesson_vo_manifest.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K115"/>
+  <dimension ref="A1:K122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2413,12 +2413,12 @@
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
-          <t>correct answer</t>
+          <t>correct answer - first try</t>
         </is>
       </c>
       <c r="H41" s="14" t="inlineStr">
         <is>
-          <t>the answer goes into the ?; confetti</t>
+          <t>a right answer at the first try: the answer goes into the ?; confetti; the equation's parts light on their words</t>
         </is>
       </c>
       <c r="I41" s="14" t="inlineStr"/>
@@ -3197,12 +3197,12 @@
       </c>
       <c r="G57" s="14" t="inlineStr">
         <is>
-          <t>correct answer</t>
+          <t>correct answer - first try</t>
         </is>
       </c>
       <c r="H57" s="14" t="inlineStr">
         <is>
-          <t>the answer goes into the ?; confetti</t>
+          <t>a right answer at the first try: the answer goes into the ?; confetti; the equation's parts light on their words</t>
         </is>
       </c>
       <c r="I57" s="14" t="inlineStr"/>
@@ -3221,44 +3221,44 @@
       </c>
       <c r="B58" s="17" t="inlineStr">
         <is>
-          <t>Page 5</t>
+          <t>Page 4</t>
         </is>
       </c>
       <c r="C58" s="18" t="inlineStr">
         <is>
-          <t>G3 · PV_SUB  (58 − 30)</t>
+          <t>G2 · PV_SUB  (47 − 20)</t>
         </is>
       </c>
       <c r="D58" s="16" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E58" s="17" t="inlineStr">
         <is>
-          <t>vo_g3_prompt</t>
+          <t>vo_g2_correct_plain</t>
         </is>
       </c>
       <c r="F58" s="19" t="inlineStr">
         <is>
-          <t>58 में से 30 घटाइए।</t>
+          <t>47 घटा 20 बराबर 27।</t>
         </is>
       </c>
       <c r="G58" s="18" t="inlineStr">
         <is>
-          <t>page instruction</t>
+          <t>correct answer - after a wrong try</t>
         </is>
       </c>
       <c r="H58" s="18" t="inlineStr">
         <is>
-          <t>as the page opens (the speaker replays it)</t>
+          <t>the same line without «शाबाश!» (cut from it - not recorded separately), after 1-3 wrong tries</t>
         </is>
       </c>
       <c r="I58" s="18" t="inlineStr"/>
       <c r="J58" s="16" t="n">
-        <v>2.51</v>
+        <v>3.82</v>
       </c>
       <c r="K58" s="17" t="inlineStr">
         <is>
-          <t>Recorded (2026-10-27)</t>
+          <t>Cut from vo_g2_correct (tools/make_plain_correct.py)</t>
         </is>
       </c>
     </row>
@@ -3277,31 +3277,31 @@
         </is>
       </c>
       <c r="D59" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E59" s="13" t="inlineStr">
         <is>
-          <t>vo_g3_sub</t>
+          <t>vo_g3_prompt</t>
         </is>
       </c>
       <c r="F59" s="15" t="inlineStr">
         <is>
-          <t>30 में 3 दहाई और 0 इकाई होती हैं।</t>
+          <t>58 में से 30 घटाइए।</t>
         </is>
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
-          <t>what is taken away</t>
+          <t>page instruction</t>
         </is>
       </c>
       <c r="H59" s="14" t="inlineStr">
         <is>
-          <t>after the build (or the opening): the number pops, its digits light on «… दहाई» / «… इकाई»; on «इसमें» the whole table lights</t>
+          <t>as the page opens (the speaker replays it)</t>
         </is>
       </c>
       <c r="I59" s="14" t="inlineStr"/>
       <c r="J59" s="12" t="n">
-        <v>4.42</v>
+        <v>2.51</v>
       </c>
       <c r="K59" s="13" t="inlineStr">
         <is>
@@ -3324,31 +3324,31 @@
         </is>
       </c>
       <c r="D60" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E60" s="17" t="inlineStr">
         <is>
-          <t>vo_g3_rm_ones0</t>
+          <t>vo_g3_sub</t>
         </is>
       </c>
       <c r="F60" s="19" t="inlineStr">
         <is>
-          <t>पहले इकाइयाँ घटाइए। 8 इकाई में से शून्य इकाई घटाते हैं।</t>
+          <t>30 में 3 दहाई और 0 इकाई होती हैं।</t>
         </is>
       </c>
       <c r="G60" s="18" t="inlineStr">
         <is>
-          <t>take-away step - the ones</t>
+          <t>what is taken away</t>
         </is>
       </c>
       <c r="H60" s="18" t="inlineStr">
         <is>
-          <t>next; the ones column beats on its «… इकाई»</t>
+          <t>after the build (or the opening): the number pops, its digits light on «… दहाई» / «… इकाई»; on «इसमें» the whole table lights</t>
         </is>
       </c>
       <c r="I60" s="18" t="inlineStr"/>
       <c r="J60" s="16" t="n">
-        <v>5.73</v>
+        <v>4.42</v>
       </c>
       <c r="K60" s="17" t="inlineStr">
         <is>
@@ -3371,35 +3371,31 @@
         </is>
       </c>
       <c r="D61" s="12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E61" s="13" t="inlineStr">
         <is>
-          <t>vo_zero</t>
+          <t>vo_g3_rm_ones0</t>
         </is>
       </c>
       <c r="F61" s="15" t="inlineStr">
         <is>
-          <t>शून्य यानी कुछ नहीं।</t>
+          <t>पहले इकाइयाँ घटाइए। 8 इकाई में से शून्य इकाई घटाते हैं।</t>
         </is>
       </c>
       <c r="G61" s="14" t="inlineStr">
         <is>
-          <t>zero ones</t>
+          <t>take-away step - the ones</t>
         </is>
       </c>
       <c r="H61" s="14" t="inlineStr">
         <is>
-          <t>straight after the ones step: no one is tappable</t>
-        </is>
-      </c>
-      <c r="I61" s="14" t="inlineStr">
-        <is>
-          <t>Page 4</t>
-        </is>
-      </c>
+          <t>next; the ones column beats on its «… इकाई»</t>
+        </is>
+      </c>
+      <c r="I61" s="14" t="inlineStr"/>
       <c r="J61" s="12" t="n">
-        <v>2.83</v>
+        <v>5.73</v>
       </c>
       <c r="K61" s="13" t="inlineStr">
         <is>
@@ -3422,31 +3418,35 @@
         </is>
       </c>
       <c r="D62" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E62" s="17" t="inlineStr">
         <is>
-          <t>vo_g3_rm_tens</t>
+          <t>vo_zero</t>
         </is>
       </c>
       <c r="F62" s="19" t="inlineStr">
         <is>
-          <t>अब दहाई घटाइए। 5 दहाई में से 3 दहाई हटाइए।</t>
+          <t>शून्य यानी कुछ नहीं।</t>
         </is>
       </c>
       <c r="G62" s="18" t="inlineStr">
         <is>
-          <t>take-away step - the tens</t>
+          <t>zero ones</t>
         </is>
       </c>
       <c r="H62" s="18" t="inlineStr">
         <is>
-          <t>when the ones are done (at once when there are none to take)</t>
-        </is>
-      </c>
-      <c r="I62" s="18" t="inlineStr"/>
+          <t>straight after the ones step: no one is tappable</t>
+        </is>
+      </c>
+      <c r="I62" s="18" t="inlineStr">
+        <is>
+          <t>Page 4</t>
+        </is>
+      </c>
       <c r="J62" s="16" t="n">
-        <v>5.25</v>
+        <v>2.83</v>
       </c>
       <c r="K62" s="17" t="inlineStr">
         <is>
@@ -3469,35 +3469,31 @@
         </is>
       </c>
       <c r="D63" s="12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E63" s="13" t="inlineStr">
         <is>
-          <t>vo_idle_rm_t</t>
+          <t>vo_g3_rm_tens</t>
         </is>
       </c>
       <c r="F63" s="15" t="inlineStr">
         <is>
-          <t>अब दहाई हटाइए।</t>
+          <t>अब दहाई घटाइए। 5 दहाई में से 3 दहाई हटाइए।</t>
         </is>
       </c>
       <c r="G63" s="14" t="inlineStr">
         <is>
-          <t>inactivity reminder - taking away</t>
+          <t>take-away step - the tens</t>
         </is>
       </c>
       <c r="H63" s="14" t="inlineStr">
         <is>
-          <t>after 7s with no tap at the take-away step, again every 7s while idle</t>
-        </is>
-      </c>
-      <c r="I63" s="14" t="inlineStr">
-        <is>
-          <t>Page 2, Page 3, Page 4, Page 6, Page 7, Page 8</t>
-        </is>
-      </c>
+          <t>when the ones are done (at once when there are none to take)</t>
+        </is>
+      </c>
+      <c r="I63" s="14" t="inlineStr"/>
       <c r="J63" s="12" t="n">
-        <v>2.2</v>
+        <v>5.25</v>
       </c>
       <c r="K63" s="13" t="inlineStr">
         <is>
@@ -3520,35 +3516,35 @@
         </is>
       </c>
       <c r="D64" s="16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E64" s="17" t="inlineStr">
         <is>
-          <t>vo_rm_tens_more</t>
+          <t>vo_idle_rm_t</t>
         </is>
       </c>
       <c r="F64" s="19" t="inlineStr">
         <is>
-          <t>आपने दहाई में ज़्यादा हटाए हैं। दोबारा कोशिश करिए।</t>
+          <t>अब दहाई हटाइए।</t>
         </is>
       </c>
       <c r="G64" s="18" t="inlineStr">
         <is>
-          <t>take-away mistake - 1st time</t>
+          <t>inactivity reminder - taking away</t>
         </is>
       </c>
       <c r="H64" s="18" t="inlineStr">
         <is>
-          <t>a ten too many taken: the tens go back, this line</t>
+          <t>after 7s with no tap at the take-away step, again every 7s while idle</t>
         </is>
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Page 3, Page 4, Page 6, Page 7, Page 8</t>
+          <t>Page 2, Page 3, Page 4, Page 6, Page 7, Page 8</t>
         </is>
       </c>
       <c r="J64" s="16" t="n">
-        <v>4.55</v>
+        <v>2.2</v>
       </c>
       <c r="K64" s="17" t="inlineStr">
         <is>
@@ -3571,26 +3567,26 @@
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E65" s="13" t="inlineStr">
         <is>
-          <t>vo_rm_guide</t>
+          <t>vo_rm_tens_more</t>
         </is>
       </c>
       <c r="F65" s="15" t="inlineStr">
         <is>
-          <t>सिर्फ़ इतने हटाइए।</t>
+          <t>आपने दहाई में ज़्यादा हटाए हैं। दोबारा कोशिश करिए।</t>
         </is>
       </c>
       <c r="G65" s="14" t="inlineStr">
         <is>
-          <t>take-away mistake - 2nd time</t>
+          <t>take-away mistake - 1st time</t>
         </is>
       </c>
       <c r="H65" s="14" t="inlineStr">
         <is>
-          <t>the tens go back; only the tens to take stay live, the others dimmed</t>
+          <t>a ten too many taken: the tens go back, this line</t>
         </is>
       </c>
       <c r="I65" s="14" t="inlineStr">
@@ -3599,7 +3595,7 @@
         </is>
       </c>
       <c r="J65" s="12" t="n">
-        <v>2.1</v>
+        <v>4.55</v>
       </c>
       <c r="K65" s="13" t="inlineStr">
         <is>
@@ -3622,35 +3618,35 @@
         </is>
       </c>
       <c r="D66" s="16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E66" s="17" t="inlineStr">
         <is>
-          <t>vo_ask_pick</t>
+          <t>vo_rm_guide</t>
         </is>
       </c>
       <c r="F66" s="19" t="inlineStr">
         <is>
-          <t>अब कितने बचे? सही संख्या चुनिए।</t>
+          <t>सिर्फ़ इतने हटाइए।</t>
         </is>
       </c>
       <c r="G66" s="18" t="inlineStr">
         <is>
-          <t>the answer question</t>
+          <t>take-away mistake - 2nd time</t>
         </is>
       </c>
       <c r="H66" s="18" t="inlineStr">
         <is>
-          <t>when the take-away is done; the cards / the keypad come in (said again after 7s idle)</t>
+          <t>the tens go back; only the tens to take stay live, the others dimmed</t>
         </is>
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>Page 4, Page 8</t>
+          <t>Page 3, Page 4, Page 6, Page 7, Page 8</t>
         </is>
       </c>
       <c r="J66" s="16" t="n">
-        <v>3.55</v>
+        <v>2.1</v>
       </c>
       <c r="K66" s="17" t="inlineStr">
         <is>
@@ -3673,35 +3669,35 @@
         </is>
       </c>
       <c r="D67" s="12" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E67" s="13" t="inlineStr">
         <is>
-          <t>vo_h_recount</t>
+          <t>vo_ask_pick</t>
         </is>
       </c>
       <c r="F67" s="15" t="inlineStr">
         <is>
-          <t>बची हुई दहाई और इकाई को दोबारा गिनिए।</t>
+          <t>अब कितने बचे? सही संख्या चुनिए।</t>
         </is>
       </c>
       <c r="G67" s="14" t="inlineStr">
         <is>
-          <t>Hint 1 (1st wrong answer)</t>
+          <t>the answer question</t>
         </is>
       </c>
       <c r="H67" s="14" t="inlineStr">
         <is>
-          <t>the columns beat on «दहाई» / «इकाई»</t>
+          <t>when the take-away is done; the cards / the keypad come in (said again after 7s idle)</t>
         </is>
       </c>
       <c r="I67" s="14" t="inlineStr">
         <is>
-          <t>Page 4, Page 6, Page 7, Page 8</t>
+          <t>Page 4, Page 8</t>
         </is>
       </c>
       <c r="J67" s="12" t="n">
-        <v>3.46</v>
+        <v>3.55</v>
       </c>
       <c r="K67" s="13" t="inlineStr">
         <is>
@@ -3724,31 +3720,35 @@
         </is>
       </c>
       <c r="D68" s="16" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E68" s="17" t="inlineStr">
         <is>
-          <t>vo_g3_h2</t>
+          <t>vo_h_recount</t>
         </is>
       </c>
       <c r="F68" s="19" t="inlineStr">
         <is>
-          <t>58 में से 30 घटाने पर, 2 दहाई और 8 इकाई बचती हैं।</t>
+          <t>बची हुई दहाई और इकाई को दोबारा गिनिए।</t>
         </is>
       </c>
       <c r="G68" s="18" t="inlineStr">
         <is>
-          <t>Hint 2 (2nd wrong answer)</t>
+          <t>Hint 1 (1st wrong answer)</t>
         </is>
       </c>
       <c r="H68" s="18" t="inlineStr">
         <is>
-          <t>the numbers light; the tens and ones left beat on their words</t>
-        </is>
-      </c>
-      <c r="I68" s="18" t="inlineStr"/>
+          <t>the columns beat on «दहाई» / «इकाई»</t>
+        </is>
+      </c>
+      <c r="I68" s="18" t="inlineStr">
+        <is>
+          <t>Page 4, Page 6, Page 7, Page 8</t>
+        </is>
+      </c>
       <c r="J68" s="16" t="n">
-        <v>6.1</v>
+        <v>3.46</v>
       </c>
       <c r="K68" s="17" t="inlineStr">
         <is>
@@ -3771,31 +3771,31 @@
         </is>
       </c>
       <c r="D69" s="12" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E69" s="13" t="inlineStr">
         <is>
-          <t>vo_g3_reveal</t>
+          <t>vo_g3_h2</t>
         </is>
       </c>
       <c r="F69" s="15" t="inlineStr">
         <is>
-          <t>58 में से 30 घटाने पर 28 बचता है। तो सही संख्या यह है।</t>
+          <t>58 में से 30 घटाने पर, 2 दहाई और 8 इकाई बचती हैं।</t>
         </is>
       </c>
       <c r="G69" s="14" t="inlineStr">
         <is>
-          <t>Hint 3 (3rd wrong answer)</t>
+          <t>Hint 2 (2nd wrong answer)</t>
         </is>
       </c>
       <c r="H69" s="14" t="inlineStr">
         <is>
-          <t>the right card / the right keys lit (one key at a time), the others off</t>
+          <t>the numbers light; the tens and ones left beat on their words</t>
         </is>
       </c>
       <c r="I69" s="14" t="inlineStr"/>
       <c r="J69" s="12" t="n">
-        <v>5.98</v>
+        <v>6.1</v>
       </c>
       <c r="K69" s="13" t="inlineStr">
         <is>
@@ -3818,80 +3818,80 @@
         </is>
       </c>
       <c r="D70" s="16" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E70" s="17" t="inlineStr">
         <is>
-          <t>vo_g3_correct</t>
+          <t>vo_g3_reveal</t>
         </is>
       </c>
       <c r="F70" s="19" t="inlineStr">
         <is>
-          <t>शाबाश! 58 घटा 30 बराबर 28।</t>
+          <t>58 में से 30 घटाने पर 28 बचता है। तो सही संख्या यह है।</t>
         </is>
       </c>
       <c r="G70" s="18" t="inlineStr">
         <is>
-          <t>correct answer</t>
+          <t>Hint 3 (3rd wrong answer)</t>
         </is>
       </c>
       <c r="H70" s="18" t="inlineStr">
         <is>
-          <t>the answer goes into the ?; confetti</t>
+          <t>the right card / the right keys lit (one key at a time), the others off</t>
         </is>
       </c>
       <c r="I70" s="18" t="inlineStr"/>
       <c r="J70" s="16" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="K70" s="17" t="inlineStr">
+        <is>
+          <t>Recorded (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>Page 5</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>G3 · PV_SUB  (58 − 30)</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="E71" s="13" t="inlineStr">
+        <is>
+          <t>vo_g3_correct</t>
+        </is>
+      </c>
+      <c r="F71" s="15" t="inlineStr">
+        <is>
+          <t>शाबाश! 58 घटा 30 बराबर 28।</t>
+        </is>
+      </c>
+      <c r="G71" s="14" t="inlineStr">
+        <is>
+          <t>correct answer - first try</t>
+        </is>
+      </c>
+      <c r="H71" s="14" t="inlineStr">
+        <is>
+          <t>a right answer at the first try: the answer goes into the ?; confetti; the equation's parts light on their words</t>
+        </is>
+      </c>
+      <c r="I71" s="14" t="inlineStr"/>
+      <c r="J71" s="12" t="n">
         <v>4.75</v>
       </c>
-      <c r="K70" s="17" t="inlineStr">
-        <is>
-          <t>Recorded (2026-10-27)</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="n">
-        <v>67</v>
-      </c>
-      <c r="B71" s="9" t="inlineStr">
-        <is>
-          <t>Transition 3</t>
-        </is>
-      </c>
-      <c r="C71" s="10" t="inlineStr">
-        <is>
-          <t>before page 6</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="9" t="inlineStr">
-        <is>
-          <t>vo_pt_practice</t>
-        </is>
-      </c>
-      <c r="F71" s="11" t="inlineStr">
-        <is>
-          <t>वाह! अब आपकी बारी।</t>
-        </is>
-      </c>
-      <c r="G71" s="10" t="inlineStr">
-        <is>
-          <t>transition line</t>
-        </is>
-      </c>
-      <c r="H71" s="10" t="inlineStr">
-        <is>
-          <t>Swiftee rises talking; «अब आपकी बारी!» wipes in as it is said</t>
-        </is>
-      </c>
-      <c r="I71" s="10" t="inlineStr"/>
-      <c r="J71" s="8" t="n">
-        <v>2.72</v>
-      </c>
-      <c r="K71" s="9" t="inlineStr">
+      <c r="K71" s="13" t="inlineStr">
         <is>
           <t>Recorded (2026-10-27)</t>
         </is>
@@ -3903,89 +3903,89 @@
       </c>
       <c r="B72" s="17" t="inlineStr">
         <is>
-          <t>Page 6</t>
+          <t>Page 5</t>
         </is>
       </c>
       <c r="C72" s="18" t="inlineStr">
         <is>
-          <t>P1 · PV_SUB  (79 − 34)</t>
+          <t>G3 · PV_SUB  (58 − 30)</t>
         </is>
       </c>
       <c r="D72" s="16" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E72" s="17" t="inlineStr">
         <is>
-          <t>vo_p1_prompt</t>
+          <t>vo_g3_correct_plain</t>
         </is>
       </c>
       <c r="F72" s="19" t="inlineStr">
         <is>
-          <t>79 में से 34 घटाइए।</t>
+          <t>58 घटा 30 बराबर 28।</t>
         </is>
       </c>
       <c r="G72" s="18" t="inlineStr">
         <is>
-          <t>page instruction</t>
+          <t>correct answer - after a wrong try</t>
         </is>
       </c>
       <c r="H72" s="18" t="inlineStr">
         <is>
-          <t>as the page opens (the speaker replays it)</t>
+          <t>the same line without «शाबाश!» (cut from it - not recorded separately), after 1-3 wrong tries</t>
         </is>
       </c>
       <c r="I72" s="18" t="inlineStr"/>
       <c r="J72" s="16" t="n">
-        <v>2.9</v>
+        <v>3.61</v>
       </c>
       <c r="K72" s="17" t="inlineStr">
         <is>
-          <t>Recorded (2026-10-27)</t>
+          <t>Cut from vo_g3_correct (tools/make_plain_correct.py)</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="12" t="n">
+      <c r="A73" s="8" t="n">
         <v>69</v>
       </c>
-      <c r="B73" s="13" t="inlineStr">
-        <is>
-          <t>Page 6</t>
-        </is>
-      </c>
-      <c r="C73" s="14" t="inlineStr">
-        <is>
-          <t>P1 · PV_SUB  (79 − 34)</t>
-        </is>
-      </c>
-      <c r="D73" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" s="13" t="inlineStr">
-        <is>
-          <t>vo_p1_rm_ones</t>
-        </is>
-      </c>
-      <c r="F73" s="15" t="inlineStr">
-        <is>
-          <t>पहले इकाई घटाइए, फिर दहाई घटाइए।</t>
-        </is>
-      </c>
-      <c r="G73" s="14" t="inlineStr">
-        <is>
-          <t>take-away instruction</t>
-        </is>
-      </c>
-      <c r="H73" s="14" t="inlineStr">
-        <is>
-          <t>next; the ones column beats on its «… इकाई», the tens on «… दहाई»; then «अब इकाई हटाइए।»</t>
-        </is>
-      </c>
-      <c r="I73" s="14" t="inlineStr"/>
-      <c r="J73" s="12" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="K73" s="13" t="inlineStr">
+      <c r="B73" s="9" t="inlineStr">
+        <is>
+          <t>Transition 3</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>before page 6</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>vo_pt_practice</t>
+        </is>
+      </c>
+      <c r="F73" s="11" t="inlineStr">
+        <is>
+          <t>वाह! अब आपकी बारी।</t>
+        </is>
+      </c>
+      <c r="G73" s="10" t="inlineStr">
+        <is>
+          <t>transition line</t>
+        </is>
+      </c>
+      <c r="H73" s="10" t="inlineStr">
+        <is>
+          <t>Swiftee rises talking; «अब आपकी बारी!» wipes in as it is said</t>
+        </is>
+      </c>
+      <c r="I73" s="10" t="inlineStr"/>
+      <c r="J73" s="8" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="K73" s="9" t="inlineStr">
         <is>
           <t>Recorded (2026-10-27)</t>
         </is>
@@ -4006,35 +4006,31 @@
         </is>
       </c>
       <c r="D74" s="16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E74" s="17" t="inlineStr">
         <is>
-          <t>vo_idle_rm_o</t>
+          <t>vo_p1_prompt</t>
         </is>
       </c>
       <c r="F74" s="19" t="inlineStr">
         <is>
-          <t>अब इकाई हटाइए।</t>
+          <t>79 में से 34 घटाइए।</t>
         </is>
       </c>
       <c r="G74" s="18" t="inlineStr">
         <is>
-          <t>take-away step said at once</t>
+          <t>page instruction</t>
         </is>
       </c>
       <c r="H74" s="18" t="inlineStr">
         <is>
-          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
-        </is>
-      </c>
-      <c r="I74" s="18" t="inlineStr">
-        <is>
-          <t>Page 3, Page 7, Page 8</t>
-        </is>
-      </c>
+          <t>as the page opens (the speaker replays it)</t>
+        </is>
+      </c>
+      <c r="I74" s="18" t="inlineStr"/>
       <c r="J74" s="16" t="n">
-        <v>2.15</v>
+        <v>2.9</v>
       </c>
       <c r="K74" s="17" t="inlineStr">
         <is>
@@ -4057,35 +4053,31 @@
         </is>
       </c>
       <c r="D75" s="12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E75" s="13" t="inlineStr">
         <is>
-          <t>vo_idle_rm_t</t>
+          <t>vo_p1_rm_ones</t>
         </is>
       </c>
       <c r="F75" s="15" t="inlineStr">
         <is>
-          <t>अब दहाई हटाइए।</t>
+          <t>पहले इकाई घटाइए, फिर दहाई घटाइए।</t>
         </is>
       </c>
       <c r="G75" s="14" t="inlineStr">
         <is>
-          <t>take-away step said at once</t>
+          <t>take-away instruction</t>
         </is>
       </c>
       <c r="H75" s="14" t="inlineStr">
         <is>
-          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
-        </is>
-      </c>
-      <c r="I75" s="14" t="inlineStr">
-        <is>
-          <t>Page 2, Page 3, Page 4, Page 5, Page 7, Page 8</t>
-        </is>
-      </c>
+          <t>next; the ones column beats on its «… इकाई», the tens on «… दहाई»; then «अब इकाई हटाइए।»</t>
+        </is>
+      </c>
+      <c r="I75" s="14" t="inlineStr"/>
       <c r="J75" s="12" t="n">
-        <v>2.2</v>
+        <v>3.69</v>
       </c>
       <c r="K75" s="13" t="inlineStr">
         <is>
@@ -4108,35 +4100,35 @@
         </is>
       </c>
       <c r="D76" s="16" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E76" s="17" t="inlineStr">
         <is>
-          <t>vo_rm_tens_more</t>
+          <t>vo_idle_rm_o</t>
         </is>
       </c>
       <c r="F76" s="19" t="inlineStr">
         <is>
-          <t>आपने दहाई में ज़्यादा हटाए हैं। दोबारा कोशिश करिए।</t>
+          <t>अब इकाई हटाइए।</t>
         </is>
       </c>
       <c r="G76" s="18" t="inlineStr">
         <is>
-          <t>take-away mistake - 1st time</t>
+          <t>take-away step said at once</t>
         </is>
       </c>
       <c r="H76" s="18" t="inlineStr">
         <is>
-          <t>a ten too many taken: the tens go back, this line</t>
+          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
         </is>
       </c>
       <c r="I76" s="18" t="inlineStr">
         <is>
-          <t>Page 3, Page 4, Page 5, Page 7, Page 8</t>
+          <t>Page 3, Page 7, Page 8</t>
         </is>
       </c>
       <c r="J76" s="16" t="n">
-        <v>4.55</v>
+        <v>2.15</v>
       </c>
       <c r="K76" s="17" t="inlineStr">
         <is>
@@ -4159,35 +4151,35 @@
         </is>
       </c>
       <c r="D77" s="12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E77" s="13" t="inlineStr">
         <is>
-          <t>vo_rm_guide</t>
+          <t>vo_idle_rm_t</t>
         </is>
       </c>
       <c r="F77" s="15" t="inlineStr">
         <is>
-          <t>सिर्फ़ इतने हटाइए।</t>
+          <t>अब दहाई हटाइए।</t>
         </is>
       </c>
       <c r="G77" s="14" t="inlineStr">
         <is>
-          <t>take-away mistake - 2nd time</t>
+          <t>take-away step said at once</t>
         </is>
       </c>
       <c r="H77" s="14" t="inlineStr">
         <is>
-          <t>the tens go back; only the tens to take stay live, the others dimmed</t>
+          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
         </is>
       </c>
       <c r="I77" s="14" t="inlineStr">
         <is>
-          <t>Page 3, Page 4, Page 5, Page 7, Page 8</t>
+          <t>Page 2, Page 3, Page 4, Page 5, Page 7, Page 8</t>
         </is>
       </c>
       <c r="J77" s="12" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="K77" s="13" t="inlineStr">
         <is>
@@ -4210,35 +4202,35 @@
         </is>
       </c>
       <c r="D78" s="16" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E78" s="17" t="inlineStr">
         <is>
-          <t>vo_p1_ask</t>
+          <t>vo_rm_tens_more</t>
         </is>
       </c>
       <c r="F78" s="19" t="inlineStr">
         <is>
-          <t>अब कितने बचे? इस डिब्बे पर सही संख्या टाइप करिए।</t>
+          <t>आपने दहाई में ज़्यादा हटाए हैं। दोबारा कोशिश करिए।</t>
         </is>
       </c>
       <c r="G78" s="18" t="inlineStr">
         <is>
-          <t>the answer question</t>
+          <t>take-away mistake - 1st time</t>
         </is>
       </c>
       <c r="H78" s="18" t="inlineStr">
         <is>
-          <t>when the take-away is done; the cards / the keypad come in (said again after 7s idle)</t>
+          <t>a ten too many taken: the tens go back, this line</t>
         </is>
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Page 7</t>
+          <t>Page 3, Page 4, Page 5, Page 7, Page 8</t>
         </is>
       </c>
       <c r="J78" s="16" t="n">
-        <v>4.37</v>
+        <v>4.55</v>
       </c>
       <c r="K78" s="17" t="inlineStr">
         <is>
@@ -4261,35 +4253,35 @@
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E79" s="13" t="inlineStr">
         <is>
-          <t>vo_h_recount</t>
+          <t>vo_rm_guide</t>
         </is>
       </c>
       <c r="F79" s="15" t="inlineStr">
         <is>
-          <t>बची हुई दहाई और इकाई को दोबारा गिनिए।</t>
+          <t>सिर्फ़ इतने हटाइए।</t>
         </is>
       </c>
       <c r="G79" s="14" t="inlineStr">
         <is>
-          <t>Hint 1 (1st wrong answer)</t>
+          <t>take-away mistake - 2nd time</t>
         </is>
       </c>
       <c r="H79" s="14" t="inlineStr">
         <is>
-          <t>the columns beat on «दहाई» / «इकाई»</t>
+          <t>the tens go back; only the tens to take stay live, the others dimmed</t>
         </is>
       </c>
       <c r="I79" s="14" t="inlineStr">
         <is>
-          <t>Page 4, Page 5, Page 7, Page 8</t>
+          <t>Page 3, Page 4, Page 5, Page 7, Page 8</t>
         </is>
       </c>
       <c r="J79" s="12" t="n">
-        <v>3.46</v>
+        <v>2.1</v>
       </c>
       <c r="K79" s="13" t="inlineStr">
         <is>
@@ -4312,31 +4304,35 @@
         </is>
       </c>
       <c r="D80" s="16" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E80" s="17" t="inlineStr">
         <is>
-          <t>vo_p1_h2</t>
+          <t>vo_p1_ask</t>
         </is>
       </c>
       <c r="F80" s="19" t="inlineStr">
         <is>
-          <t>79 में से 34 घटाने पर, 4 दहाई और 5 इकाई बचती हैं।</t>
+          <t>अब कितने बचे? इस डिब्बे पर सही संख्या टाइप करिए।</t>
         </is>
       </c>
       <c r="G80" s="18" t="inlineStr">
         <is>
-          <t>Hint 2 (2nd wrong answer)</t>
+          <t>the answer question</t>
         </is>
       </c>
       <c r="H80" s="18" t="inlineStr">
         <is>
-          <t>the numbers light; the tens and ones left beat on their words</t>
-        </is>
-      </c>
-      <c r="I80" s="18" t="inlineStr"/>
+          <t>when the take-away is done; the cards / the keypad come in (said again after 7s idle)</t>
+        </is>
+      </c>
+      <c r="I80" s="18" t="inlineStr">
+        <is>
+          <t>Page 7</t>
+        </is>
+      </c>
       <c r="J80" s="16" t="n">
-        <v>5.9</v>
+        <v>4.37</v>
       </c>
       <c r="K80" s="17" t="inlineStr">
         <is>
@@ -4359,31 +4355,35 @@
         </is>
       </c>
       <c r="D81" s="12" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E81" s="13" t="inlineStr">
         <is>
-          <t>vo_p1_reveal</t>
+          <t>vo_h_recount</t>
         </is>
       </c>
       <c r="F81" s="15" t="inlineStr">
         <is>
-          <t>79 में से 34 घटाने पर 45 बचता है। तो सही संख्या यह है।</t>
+          <t>बची हुई दहाई और इकाई को दोबारा गिनिए।</t>
         </is>
       </c>
       <c r="G81" s="14" t="inlineStr">
         <is>
-          <t>Hint 3 (3rd wrong answer)</t>
+          <t>Hint 1 (1st wrong answer)</t>
         </is>
       </c>
       <c r="H81" s="14" t="inlineStr">
         <is>
-          <t>the right card / the right keys lit (one key at a time), the others off</t>
-        </is>
-      </c>
-      <c r="I81" s="14" t="inlineStr"/>
+          <t>the columns beat on «दहाई» / «इकाई»</t>
+        </is>
+      </c>
+      <c r="I81" s="14" t="inlineStr">
+        <is>
+          <t>Page 4, Page 5, Page 7, Page 8</t>
+        </is>
+      </c>
       <c r="J81" s="12" t="n">
-        <v>6.83</v>
+        <v>3.46</v>
       </c>
       <c r="K81" s="13" t="inlineStr">
         <is>
@@ -4406,31 +4406,31 @@
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E82" s="17" t="inlineStr">
         <is>
-          <t>vo_p1_correct</t>
+          <t>vo_p1_h2</t>
         </is>
       </c>
       <c r="F82" s="19" t="inlineStr">
         <is>
-          <t>शाबाश! 79 घटा 34 बराबर 45।</t>
+          <t>79 में से 34 घटाने पर, 4 दहाई और 5 इकाई बचती हैं।</t>
         </is>
       </c>
       <c r="G82" s="18" t="inlineStr">
         <is>
-          <t>correct answer</t>
+          <t>Hint 2 (2nd wrong answer)</t>
         </is>
       </c>
       <c r="H82" s="18" t="inlineStr">
         <is>
-          <t>the answer goes into the ?; confetti</t>
+          <t>the numbers light; the tens and ones left beat on their words</t>
         </is>
       </c>
       <c r="I82" s="18" t="inlineStr"/>
       <c r="J82" s="16" t="n">
-        <v>6.12</v>
+        <v>5.9</v>
       </c>
       <c r="K82" s="17" t="inlineStr">
         <is>
@@ -4444,40 +4444,40 @@
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
-          <t>Page 7</t>
+          <t>Page 6</t>
         </is>
       </c>
       <c r="C83" s="14" t="inlineStr">
         <is>
-          <t>P2 · PV_SUB  (90 − 40)</t>
+          <t>P1 · PV_SUB  (79 − 34)</t>
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E83" s="13" t="inlineStr">
         <is>
-          <t>vo_p90_prompt</t>
+          <t>vo_p1_reveal</t>
         </is>
       </c>
       <c r="F83" s="15" t="inlineStr">
         <is>
-          <t>90 में से 40 घटाइए।</t>
+          <t>79 में से 34 घटाने पर 45 बचता है। तो सही संख्या यह है।</t>
         </is>
       </c>
       <c r="G83" s="14" t="inlineStr">
         <is>
-          <t>page instruction</t>
+          <t>Hint 3 (3rd wrong answer)</t>
         </is>
       </c>
       <c r="H83" s="14" t="inlineStr">
         <is>
-          <t>as the page opens (the speaker replays it)</t>
+          <t>the right card / the right keys lit (one key at a time), the others off</t>
         </is>
       </c>
       <c r="I83" s="14" t="inlineStr"/>
       <c r="J83" s="12" t="n">
-        <v>2.78</v>
+        <v>6.83</v>
       </c>
       <c r="K83" s="13" t="inlineStr">
         <is>
@@ -4491,40 +4491,40 @@
       </c>
       <c r="B84" s="17" t="inlineStr">
         <is>
-          <t>Page 7</t>
+          <t>Page 6</t>
         </is>
       </c>
       <c r="C84" s="18" t="inlineStr">
         <is>
-          <t>P2 · PV_SUB  (90 − 40)</t>
+          <t>P1 · PV_SUB  (79 − 34)</t>
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E84" s="17" t="inlineStr">
         <is>
-          <t>vo_g3_rm_ones</t>
+          <t>vo_p1_correct</t>
         </is>
       </c>
       <c r="F84" s="19" t="inlineStr">
         <is>
-          <t>पहले इकाई घटाइए, फिर दहाई घटाइए।</t>
+          <t>शाबाश! 79 घटा 34 बराबर 45।</t>
         </is>
       </c>
       <c r="G84" s="18" t="inlineStr">
         <is>
-          <t>take-away instruction</t>
+          <t>correct answer - first try</t>
         </is>
       </c>
       <c r="H84" s="18" t="inlineStr">
         <is>
-          <t>next; the ones column beats on its «… इकाई», the tens on «… दहाई»; then «अब इकाई हटाइए।»</t>
+          <t>a right answer at the first try: the answer goes into the ?; confetti; the equation's parts light on their words</t>
         </is>
       </c>
       <c r="I84" s="18" t="inlineStr"/>
       <c r="J84" s="16" t="n">
-        <v>3.82</v>
+        <v>6.12</v>
       </c>
       <c r="K84" s="17" t="inlineStr">
         <is>
@@ -4538,48 +4538,44 @@
       </c>
       <c r="B85" s="13" t="inlineStr">
         <is>
-          <t>Page 7</t>
+          <t>Page 6</t>
         </is>
       </c>
       <c r="C85" s="14" t="inlineStr">
         <is>
-          <t>P2 · PV_SUB  (90 − 40)</t>
+          <t>P1 · PV_SUB  (79 − 34)</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E85" s="13" t="inlineStr">
         <is>
-          <t>vo_idle_rm_o</t>
+          <t>vo_p1_correct_plain</t>
         </is>
       </c>
       <c r="F85" s="15" t="inlineStr">
         <is>
-          <t>अब इकाई हटाइए।</t>
+          <t>79 घटा 34 बराबर 45।</t>
         </is>
       </c>
       <c r="G85" s="14" t="inlineStr">
         <is>
-          <t>take-away step said at once</t>
+          <t>correct answer - after a wrong try</t>
         </is>
       </c>
       <c r="H85" s="14" t="inlineStr">
         <is>
-          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
-        </is>
-      </c>
-      <c r="I85" s="14" t="inlineStr">
-        <is>
-          <t>Page 3, Page 6, Page 8</t>
-        </is>
-      </c>
+          <t>the same line without «शाबाश!» (cut from it - not recorded separately), after 1-3 wrong tries</t>
+        </is>
+      </c>
+      <c r="I85" s="14" t="inlineStr"/>
       <c r="J85" s="12" t="n">
-        <v>2.15</v>
+        <v>4.82</v>
       </c>
       <c r="K85" s="13" t="inlineStr">
         <is>
-          <t>Recorded (2026-10-27)</t>
+          <t>Cut from vo_p1_correct (tools/make_plain_correct.py)</t>
         </is>
       </c>
     </row>
@@ -4598,35 +4594,31 @@
         </is>
       </c>
       <c r="D86" s="16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E86" s="17" t="inlineStr">
         <is>
-          <t>vo_idle_rm_t</t>
+          <t>vo_p90_prompt</t>
         </is>
       </c>
       <c r="F86" s="19" t="inlineStr">
         <is>
-          <t>अब दहाई हटाइए।</t>
+          <t>90 में से 40 घटाइए।</t>
         </is>
       </c>
       <c r="G86" s="18" t="inlineStr">
         <is>
-          <t>take-away step said at once</t>
+          <t>page instruction</t>
         </is>
       </c>
       <c r="H86" s="18" t="inlineStr">
         <is>
-          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
-        </is>
-      </c>
-      <c r="I86" s="18" t="inlineStr">
-        <is>
-          <t>Page 2, Page 3, Page 4, Page 5, Page 6, Page 8</t>
-        </is>
-      </c>
+          <t>as the page opens (the speaker replays it)</t>
+        </is>
+      </c>
+      <c r="I86" s="18" t="inlineStr"/>
       <c r="J86" s="16" t="n">
-        <v>2.2</v>
+        <v>2.78</v>
       </c>
       <c r="K86" s="17" t="inlineStr">
         <is>
@@ -4649,35 +4641,31 @@
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E87" s="13" t="inlineStr">
         <is>
-          <t>vo_rm_tens_more</t>
+          <t>vo_g3_rm_ones</t>
         </is>
       </c>
       <c r="F87" s="15" t="inlineStr">
         <is>
-          <t>आपने दहाई में ज़्यादा हटाए हैं। दोबारा कोशिश करिए।</t>
+          <t>पहले इकाई घटाइए, फिर दहाई घटाइए।</t>
         </is>
       </c>
       <c r="G87" s="14" t="inlineStr">
         <is>
-          <t>take-away mistake - 1st time</t>
+          <t>take-away instruction</t>
         </is>
       </c>
       <c r="H87" s="14" t="inlineStr">
         <is>
-          <t>a ten too many taken: the tens go back, this line</t>
-        </is>
-      </c>
-      <c r="I87" s="14" t="inlineStr">
-        <is>
-          <t>Page 3, Page 4, Page 5, Page 6, Page 8</t>
-        </is>
-      </c>
+          <t>next; the ones column beats on its «… इकाई», the tens on «… दहाई»; then «अब इकाई हटाइए।»</t>
+        </is>
+      </c>
+      <c r="I87" s="14" t="inlineStr"/>
       <c r="J87" s="12" t="n">
-        <v>4.55</v>
+        <v>3.82</v>
       </c>
       <c r="K87" s="13" t="inlineStr">
         <is>
@@ -4700,35 +4688,35 @@
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E88" s="17" t="inlineStr">
         <is>
-          <t>vo_rm_guide</t>
+          <t>vo_idle_rm_o</t>
         </is>
       </c>
       <c r="F88" s="19" t="inlineStr">
         <is>
-          <t>सिर्फ़ इतने हटाइए।</t>
+          <t>अब इकाई हटाइए।</t>
         </is>
       </c>
       <c r="G88" s="18" t="inlineStr">
         <is>
-          <t>take-away mistake - 2nd time</t>
+          <t>take-away step said at once</t>
         </is>
       </c>
       <c r="H88" s="18" t="inlineStr">
         <is>
-          <t>the tens go back; only the tens to take stay live, the others dimmed</t>
+          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
         </is>
       </c>
       <c r="I88" s="18" t="inlineStr">
         <is>
-          <t>Page 3, Page 4, Page 5, Page 6, Page 8</t>
+          <t>Page 3, Page 6, Page 8</t>
         </is>
       </c>
       <c r="J88" s="16" t="n">
-        <v>2.1</v>
+        <v>2.15</v>
       </c>
       <c r="K88" s="17" t="inlineStr">
         <is>
@@ -4751,35 +4739,35 @@
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E89" s="13" t="inlineStr">
         <is>
-          <t>vo_p1_ask</t>
+          <t>vo_idle_rm_t</t>
         </is>
       </c>
       <c r="F89" s="15" t="inlineStr">
         <is>
-          <t>अब कितने बचे? इस डिब्बे पर सही संख्या टाइप करिए।</t>
+          <t>अब दहाई हटाइए।</t>
         </is>
       </c>
       <c r="G89" s="14" t="inlineStr">
         <is>
-          <t>the answer question</t>
+          <t>take-away step said at once</t>
         </is>
       </c>
       <c r="H89" s="14" t="inlineStr">
         <is>
-          <t>when the take-away is done; the cards / the keypad come in (said again after 7s idle)</t>
+          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
         </is>
       </c>
       <c r="I89" s="14" t="inlineStr">
         <is>
-          <t>Page 6</t>
+          <t>Page 2, Page 3, Page 4, Page 5, Page 6, Page 8</t>
         </is>
       </c>
       <c r="J89" s="12" t="n">
-        <v>4.37</v>
+        <v>2.2</v>
       </c>
       <c r="K89" s="13" t="inlineStr">
         <is>
@@ -4802,35 +4790,35 @@
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E90" s="17" t="inlineStr">
         <is>
-          <t>vo_h_recount</t>
+          <t>vo_rm_tens_more</t>
         </is>
       </c>
       <c r="F90" s="19" t="inlineStr">
         <is>
-          <t>बची हुई दहाई और इकाई को दोबारा गिनिए।</t>
+          <t>आपने दहाई में ज़्यादा हटाए हैं। दोबारा कोशिश करिए।</t>
         </is>
       </c>
       <c r="G90" s="18" t="inlineStr">
         <is>
-          <t>Hint 1 (1st wrong answer)</t>
+          <t>take-away mistake - 1st time</t>
         </is>
       </c>
       <c r="H90" s="18" t="inlineStr">
         <is>
-          <t>the columns beat on «दहाई» / «इकाई»</t>
+          <t>a ten too many taken: the tens go back, this line</t>
         </is>
       </c>
       <c r="I90" s="18" t="inlineStr">
         <is>
-          <t>Page 4, Page 5, Page 6, Page 8</t>
+          <t>Page 3, Page 4, Page 5, Page 6, Page 8</t>
         </is>
       </c>
       <c r="J90" s="16" t="n">
-        <v>3.46</v>
+        <v>4.55</v>
       </c>
       <c r="K90" s="17" t="inlineStr">
         <is>
@@ -4853,31 +4841,35 @@
         </is>
       </c>
       <c r="D91" s="12" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E91" s="13" t="inlineStr">
         <is>
-          <t>vo_p4_h2</t>
+          <t>vo_rm_guide</t>
         </is>
       </c>
       <c r="F91" s="15" t="inlineStr">
         <is>
-          <t>90 में से 40 घटाने पर, 5 दहाई और 0 इकाई बचती हैं।</t>
+          <t>सिर्फ़ इतने हटाइए।</t>
         </is>
       </c>
       <c r="G91" s="14" t="inlineStr">
         <is>
-          <t>Hint 2 (2nd wrong answer)</t>
+          <t>take-away mistake - 2nd time</t>
         </is>
       </c>
       <c r="H91" s="14" t="inlineStr">
         <is>
-          <t>the numbers light; the tens and ones left beat on their words</t>
-        </is>
-      </c>
-      <c r="I91" s="14" t="inlineStr"/>
+          <t>the tens go back; only the tens to take stay live, the others dimmed</t>
+        </is>
+      </c>
+      <c r="I91" s="14" t="inlineStr">
+        <is>
+          <t>Page 3, Page 4, Page 5, Page 6, Page 8</t>
+        </is>
+      </c>
       <c r="J91" s="12" t="n">
-        <v>6</v>
+        <v>2.1</v>
       </c>
       <c r="K91" s="13" t="inlineStr">
         <is>
@@ -4900,31 +4892,35 @@
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E92" s="17" t="inlineStr">
         <is>
-          <t>vo_p4_reveal</t>
+          <t>vo_p1_ask</t>
         </is>
       </c>
       <c r="F92" s="19" t="inlineStr">
         <is>
-          <t>90 में से 40 घटाने पर 50 बचता है। तो सही संख्या यह है।</t>
+          <t>अब कितने बचे? इस डिब्बे पर सही संख्या टाइप करिए।</t>
         </is>
       </c>
       <c r="G92" s="18" t="inlineStr">
         <is>
-          <t>Hint 3 (3rd wrong answer)</t>
+          <t>the answer question</t>
         </is>
       </c>
       <c r="H92" s="18" t="inlineStr">
         <is>
-          <t>the right card / the right keys lit (one key at a time), the others off</t>
-        </is>
-      </c>
-      <c r="I92" s="18" t="inlineStr"/>
+          <t>when the take-away is done; the cards / the keypad come in (said again after 7s idle)</t>
+        </is>
+      </c>
+      <c r="I92" s="18" t="inlineStr">
+        <is>
+          <t>Page 6</t>
+        </is>
+      </c>
       <c r="J92" s="16" t="n">
-        <v>5.53</v>
+        <v>4.37</v>
       </c>
       <c r="K92" s="17" t="inlineStr">
         <is>
@@ -4947,31 +4943,35 @@
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E93" s="13" t="inlineStr">
         <is>
-          <t>vo_p90_correct</t>
+          <t>vo_h_recount</t>
         </is>
       </c>
       <c r="F93" s="15" t="inlineStr">
         <is>
-          <t>शाबाश! 90 घटा 40 बराबर 50।</t>
+          <t>बची हुई दहाई और इकाई को दोबारा गिनिए।</t>
         </is>
       </c>
       <c r="G93" s="14" t="inlineStr">
         <is>
-          <t>correct answer</t>
+          <t>Hint 1 (1st wrong answer)</t>
         </is>
       </c>
       <c r="H93" s="14" t="inlineStr">
         <is>
-          <t>the answer goes into the ?; confetti</t>
-        </is>
-      </c>
-      <c r="I93" s="14" t="inlineStr"/>
+          <t>the columns beat on «दहाई» / «इकाई»</t>
+        </is>
+      </c>
+      <c r="I93" s="14" t="inlineStr">
+        <is>
+          <t>Page 4, Page 5, Page 6, Page 8</t>
+        </is>
+      </c>
       <c r="J93" s="12" t="n">
-        <v>4.92</v>
+        <v>3.46</v>
       </c>
       <c r="K93" s="13" t="inlineStr">
         <is>
@@ -4985,40 +4985,40 @@
       </c>
       <c r="B94" s="17" t="inlineStr">
         <is>
-          <t>Page 8</t>
+          <t>Page 7</t>
         </is>
       </c>
       <c r="C94" s="18" t="inlineStr">
         <is>
-          <t>P3 · PV_SUB  (86 − 56)</t>
+          <t>P2 · PV_SUB  (90 − 40)</t>
         </is>
       </c>
       <c r="D94" s="16" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E94" s="17" t="inlineStr">
         <is>
-          <t>vo_p2_prompt</t>
+          <t>vo_p4_h2</t>
         </is>
       </c>
       <c r="F94" s="19" t="inlineStr">
         <is>
-          <t>86 में से 56 घटाइए और फिर सही संख्या चुनिए।</t>
+          <t>90 में से 40 घटाने पर, 5 दहाई और 0 इकाई बचती हैं।</t>
         </is>
       </c>
       <c r="G94" s="18" t="inlineStr">
         <is>
-          <t>page instruction</t>
+          <t>Hint 2 (2nd wrong answer)</t>
         </is>
       </c>
       <c r="H94" s="18" t="inlineStr">
         <is>
-          <t>as the page opens (the speaker replays it)</t>
+          <t>the numbers light; the tens and ones left beat on their words</t>
         </is>
       </c>
       <c r="I94" s="18" t="inlineStr"/>
       <c r="J94" s="16" t="n">
-        <v>4.53</v>
+        <v>6</v>
       </c>
       <c r="K94" s="17" t="inlineStr">
         <is>
@@ -5032,40 +5032,40 @@
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
-          <t>Page 8</t>
+          <t>Page 7</t>
         </is>
       </c>
       <c r="C95" s="14" t="inlineStr">
         <is>
-          <t>P3 · PV_SUB  (86 − 56)</t>
+          <t>P2 · PV_SUB  (90 − 40)</t>
         </is>
       </c>
       <c r="D95" s="12" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E95" s="13" t="inlineStr">
         <is>
-          <t>vo_p2_remove</t>
+          <t>vo_p4_reveal</t>
         </is>
       </c>
       <c r="F95" s="15" t="inlineStr">
         <is>
-          <t>दिए हुए ब्लॉक्स पर टैप करके 56 ब्लॉक्स हटाइए। पहले इकाई में से हटाइए, फिर दहाई में से।</t>
+          <t>90 में से 40 घटाने पर 50 बचता है। तो सही संख्या यह है।</t>
         </is>
       </c>
       <c r="G95" s="14" t="inlineStr">
         <is>
-          <t>take-away instruction</t>
+          <t>Hint 3 (3rd wrong answer)</t>
         </is>
       </c>
       <c r="H95" s="14" t="inlineStr">
         <is>
-          <t>next; the ones column beats on its «… इकाई», the tens on «… दहाई»; then «अब इकाई हटाइए।»</t>
+          <t>the right card / the right keys lit (one key at a time), the others off</t>
         </is>
       </c>
       <c r="I95" s="14" t="inlineStr"/>
       <c r="J95" s="12" t="n">
-        <v>8.34</v>
+        <v>5.53</v>
       </c>
       <c r="K95" s="13" t="inlineStr">
         <is>
@@ -5079,44 +5079,40 @@
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>Page 8</t>
+          <t>Page 7</t>
         </is>
       </c>
       <c r="C96" s="18" t="inlineStr">
         <is>
-          <t>P3 · PV_SUB  (86 − 56)</t>
+          <t>P2 · PV_SUB  (90 − 40)</t>
         </is>
       </c>
       <c r="D96" s="16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E96" s="17" t="inlineStr">
         <is>
-          <t>vo_idle_rm_o</t>
+          <t>vo_p90_correct</t>
         </is>
       </c>
       <c r="F96" s="19" t="inlineStr">
         <is>
-          <t>अब इकाई हटाइए।</t>
+          <t>शाबाश! 90 घटा 40 बराबर 50।</t>
         </is>
       </c>
       <c r="G96" s="18" t="inlineStr">
         <is>
-          <t>take-away step said at once</t>
+          <t>correct answer - first try</t>
         </is>
       </c>
       <c r="H96" s="18" t="inlineStr">
         <is>
-          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
-        </is>
-      </c>
-      <c r="I96" s="18" t="inlineStr">
-        <is>
-          <t>Page 3, Page 6, Page 7</t>
-        </is>
-      </c>
+          <t>a right answer at the first try: the answer goes into the ?; confetti; the equation's parts light on their words</t>
+        </is>
+      </c>
+      <c r="I96" s="18" t="inlineStr"/>
       <c r="J96" s="16" t="n">
-        <v>2.15</v>
+        <v>4.92</v>
       </c>
       <c r="K96" s="17" t="inlineStr">
         <is>
@@ -5130,48 +5126,44 @@
       </c>
       <c r="B97" s="13" t="inlineStr">
         <is>
-          <t>Page 8</t>
+          <t>Page 7</t>
         </is>
       </c>
       <c r="C97" s="14" t="inlineStr">
         <is>
-          <t>P3 · PV_SUB  (86 − 56)</t>
+          <t>P2 · PV_SUB  (90 − 40)</t>
         </is>
       </c>
       <c r="D97" s="12" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E97" s="13" t="inlineStr">
         <is>
-          <t>vo_idle_rm_t</t>
+          <t>vo_p90_correct_plain</t>
         </is>
       </c>
       <c r="F97" s="15" t="inlineStr">
         <is>
-          <t>अब दहाई हटाइए।</t>
+          <t>90 घटा 40 बराबर 50।</t>
         </is>
       </c>
       <c r="G97" s="14" t="inlineStr">
         <is>
-          <t>take-away step said at once</t>
+          <t>correct answer - after a wrong try</t>
         </is>
       </c>
       <c r="H97" s="14" t="inlineStr">
         <is>
-          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
-        </is>
-      </c>
-      <c r="I97" s="14" t="inlineStr">
-        <is>
-          <t>Page 2, Page 3, Page 4, Page 5, Page 6, Page 7</t>
-        </is>
-      </c>
+          <t>the same line without «शाबाश!» (cut from it - not recorded separately), after 1-3 wrong tries</t>
+        </is>
+      </c>
+      <c r="I97" s="14" t="inlineStr"/>
       <c r="J97" s="12" t="n">
-        <v>2.2</v>
+        <v>3.52</v>
       </c>
       <c r="K97" s="13" t="inlineStr">
         <is>
-          <t>Recorded (2026-10-27)</t>
+          <t>Cut from vo_p90_correct (tools/make_plain_correct.py)</t>
         </is>
       </c>
     </row>
@@ -5190,35 +5182,31 @@
         </is>
       </c>
       <c r="D98" s="16" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E98" s="17" t="inlineStr">
         <is>
-          <t>vo_rm_tens_more</t>
+          <t>vo_p2_prompt</t>
         </is>
       </c>
       <c r="F98" s="19" t="inlineStr">
         <is>
-          <t>आपने दहाई में ज़्यादा हटाए हैं। दोबारा कोशिश करिए।</t>
+          <t>86 में से 56 घटाइए और फिर सही संख्या चुनिए।</t>
         </is>
       </c>
       <c r="G98" s="18" t="inlineStr">
         <is>
-          <t>take-away mistake - 1st time</t>
+          <t>page instruction</t>
         </is>
       </c>
       <c r="H98" s="18" t="inlineStr">
         <is>
-          <t>a ten too many taken: the tens go back, this line</t>
-        </is>
-      </c>
-      <c r="I98" s="18" t="inlineStr">
-        <is>
-          <t>Page 3, Page 4, Page 5, Page 6, Page 7</t>
-        </is>
-      </c>
+          <t>as the page opens (the speaker replays it)</t>
+        </is>
+      </c>
+      <c r="I98" s="18" t="inlineStr"/>
       <c r="J98" s="16" t="n">
-        <v>4.55</v>
+        <v>4.53</v>
       </c>
       <c r="K98" s="17" t="inlineStr">
         <is>
@@ -5241,35 +5229,31 @@
         </is>
       </c>
       <c r="D99" s="12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E99" s="13" t="inlineStr">
         <is>
-          <t>vo_rm_guide</t>
+          <t>vo_p2_remove</t>
         </is>
       </c>
       <c r="F99" s="15" t="inlineStr">
         <is>
-          <t>सिर्फ़ इतने हटाइए।</t>
+          <t>दिए हुए ब्लॉक्स पर टैप करके 56 ब्लॉक्स हटाइए। पहले इकाई में से हटाइए, फिर दहाई में से।</t>
         </is>
       </c>
       <c r="G99" s="14" t="inlineStr">
         <is>
-          <t>take-away mistake - 2nd time</t>
+          <t>take-away instruction</t>
         </is>
       </c>
       <c r="H99" s="14" t="inlineStr">
         <is>
-          <t>the tens go back; only the tens to take stay live, the others dimmed</t>
-        </is>
-      </c>
-      <c r="I99" s="14" t="inlineStr">
-        <is>
-          <t>Page 3, Page 4, Page 5, Page 6, Page 7</t>
-        </is>
-      </c>
+          <t>next; the ones column beats on its «… इकाई», the tens on «… दहाई»; then «अब इकाई हटाइए।»</t>
+        </is>
+      </c>
+      <c r="I99" s="14" t="inlineStr"/>
       <c r="J99" s="12" t="n">
-        <v>2.1</v>
+        <v>8.34</v>
       </c>
       <c r="K99" s="13" t="inlineStr">
         <is>
@@ -5292,35 +5276,35 @@
         </is>
       </c>
       <c r="D100" s="16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E100" s="17" t="inlineStr">
         <is>
-          <t>vo_ask_pick</t>
+          <t>vo_idle_rm_o</t>
         </is>
       </c>
       <c r="F100" s="19" t="inlineStr">
         <is>
-          <t>अब कितने बचे? सही संख्या चुनिए।</t>
+          <t>अब इकाई हटाइए।</t>
         </is>
       </c>
       <c r="G100" s="18" t="inlineStr">
         <is>
-          <t>the answer question</t>
+          <t>take-away step said at once</t>
         </is>
       </c>
       <c r="H100" s="18" t="inlineStr">
         <is>
-          <t>when the take-away is done; the cards / the keypad come in (said again after 7s idle)</t>
+          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
         </is>
       </c>
       <c r="I100" s="18" t="inlineStr">
         <is>
-          <t>Page 4, Page 5</t>
+          <t>Page 3, Page 6, Page 7</t>
         </is>
       </c>
       <c r="J100" s="16" t="n">
-        <v>3.55</v>
+        <v>2.15</v>
       </c>
       <c r="K100" s="17" t="inlineStr">
         <is>
@@ -5343,35 +5327,35 @@
         </is>
       </c>
       <c r="D101" s="12" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E101" s="13" t="inlineStr">
         <is>
-          <t>vo_h_recount</t>
+          <t>vo_idle_rm_t</t>
         </is>
       </c>
       <c r="F101" s="15" t="inlineStr">
         <is>
-          <t>बची हुई दहाई और इकाई को दोबारा गिनिए।</t>
+          <t>अब दहाई हटाइए।</t>
         </is>
       </c>
       <c r="G101" s="14" t="inlineStr">
         <is>
-          <t>Hint 1 (1st wrong answer)</t>
+          <t>take-away step said at once</t>
         </is>
       </c>
       <c r="H101" s="14" t="inlineStr">
         <is>
-          <t>the columns beat on «दहाई» / «इकाई»</t>
+          <t>on a page with one take-away line: «अब इकाई हटाइए।» right after it, «अब दहाई हटाइए।» as the ones are done (tens pulse); then as the 7s reminder</t>
         </is>
       </c>
       <c r="I101" s="14" t="inlineStr">
         <is>
-          <t>Page 4, Page 5, Page 6, Page 7</t>
+          <t>Page 2, Page 3, Page 4, Page 5, Page 6, Page 7</t>
         </is>
       </c>
       <c r="J101" s="12" t="n">
-        <v>3.46</v>
+        <v>2.2</v>
       </c>
       <c r="K101" s="13" t="inlineStr">
         <is>
@@ -5394,31 +5378,35 @@
         </is>
       </c>
       <c r="D102" s="16" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E102" s="17" t="inlineStr">
         <is>
-          <t>vo_p2_h2</t>
+          <t>vo_rm_tens_more</t>
         </is>
       </c>
       <c r="F102" s="19" t="inlineStr">
         <is>
-          <t>86 में से 56 घटाने पर, 3 दहाई और 0 इकाई बचती हैं।</t>
+          <t>आपने दहाई में ज़्यादा हटाए हैं। दोबारा कोशिश करिए।</t>
         </is>
       </c>
       <c r="G102" s="18" t="inlineStr">
         <is>
-          <t>Hint 2 (2nd wrong answer)</t>
+          <t>take-away mistake - 1st time</t>
         </is>
       </c>
       <c r="H102" s="18" t="inlineStr">
         <is>
-          <t>the numbers light; the tens and ones left beat on their words</t>
-        </is>
-      </c>
-      <c r="I102" s="18" t="inlineStr"/>
+          <t>a ten too many taken: the tens go back, this line</t>
+        </is>
+      </c>
+      <c r="I102" s="18" t="inlineStr">
+        <is>
+          <t>Page 3, Page 4, Page 5, Page 6, Page 7</t>
+        </is>
+      </c>
       <c r="J102" s="16" t="n">
-        <v>6.07</v>
+        <v>4.55</v>
       </c>
       <c r="K102" s="17" t="inlineStr">
         <is>
@@ -5441,31 +5429,35 @@
         </is>
       </c>
       <c r="D103" s="12" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E103" s="13" t="inlineStr">
         <is>
-          <t>vo_p2_reveal</t>
+          <t>vo_rm_guide</t>
         </is>
       </c>
       <c r="F103" s="15" t="inlineStr">
         <is>
-          <t>86 में से 56 घटाने पर 30 बचता है। तो सही संख्या यह है।</t>
+          <t>सिर्फ़ इतने हटाइए।</t>
         </is>
       </c>
       <c r="G103" s="14" t="inlineStr">
         <is>
-          <t>Hint 3 (3rd wrong answer)</t>
+          <t>take-away mistake - 2nd time</t>
         </is>
       </c>
       <c r="H103" s="14" t="inlineStr">
         <is>
-          <t>the right card / the right keys lit (one key at a time), the others off</t>
-        </is>
-      </c>
-      <c r="I103" s="14" t="inlineStr"/>
+          <t>the tens go back; only the tens to take stay live, the others dimmed</t>
+        </is>
+      </c>
+      <c r="I103" s="14" t="inlineStr">
+        <is>
+          <t>Page 3, Page 4, Page 5, Page 6, Page 7</t>
+        </is>
+      </c>
       <c r="J103" s="12" t="n">
-        <v>5.42</v>
+        <v>2.1</v>
       </c>
       <c r="K103" s="13" t="inlineStr">
         <is>
@@ -5488,31 +5480,35 @@
         </is>
       </c>
       <c r="D104" s="16" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E104" s="17" t="inlineStr">
         <is>
-          <t>vo_p2_correct</t>
+          <t>vo_ask_pick</t>
         </is>
       </c>
       <c r="F104" s="19" t="inlineStr">
         <is>
-          <t>शाबाश! आपने सही संख्या चुन ली। 86 घटा 56 बराबर 30।</t>
+          <t>अब कितने बचे? सही संख्या चुनिए।</t>
         </is>
       </c>
       <c r="G104" s="18" t="inlineStr">
         <is>
-          <t>correct answer</t>
+          <t>the answer question</t>
         </is>
       </c>
       <c r="H104" s="18" t="inlineStr">
         <is>
-          <t>the answer goes into the ?; confetti</t>
-        </is>
-      </c>
-      <c r="I104" s="18" t="inlineStr"/>
+          <t>when the take-away is done; the cards / the keypad come in (said again after 7s idle)</t>
+        </is>
+      </c>
+      <c r="I104" s="18" t="inlineStr">
+        <is>
+          <t>Page 4, Page 5</t>
+        </is>
+      </c>
       <c r="J104" s="16" t="n">
-        <v>7.12</v>
+        <v>3.55</v>
       </c>
       <c r="K104" s="17" t="inlineStr">
         <is>
@@ -5526,40 +5522,44 @@
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
-          <t>Page 9</t>
+          <t>Page 8</t>
         </is>
       </c>
       <c r="C105" s="14" t="inlineStr">
         <is>
-          <t>P4 · MENTAL_SUB  (45 − 12)</t>
+          <t>P3 · PV_SUB  (86 − 56)</t>
         </is>
       </c>
       <c r="D105" s="12" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E105" s="13" t="inlineStr">
         <is>
-          <t>vo_p3_prompt</t>
+          <t>vo_h_recount</t>
         </is>
       </c>
       <c r="F105" s="15" t="inlineStr">
         <is>
-          <t>45 में से 12 घटाइए और सही संख्या चुनिए।</t>
+          <t>बची हुई दहाई और इकाई को दोबारा गिनिए।</t>
         </is>
       </c>
       <c r="G105" s="14" t="inlineStr">
         <is>
-          <t>page instruction</t>
+          <t>Hint 1 (1st wrong answer)</t>
         </is>
       </c>
       <c r="H105" s="14" t="inlineStr">
         <is>
-          <t>as the page opens (the speaker replays it)</t>
-        </is>
-      </c>
-      <c r="I105" s="14" t="inlineStr"/>
+          <t>the columns beat on «दहाई» / «इकाई»</t>
+        </is>
+      </c>
+      <c r="I105" s="14" t="inlineStr">
+        <is>
+          <t>Page 4, Page 5, Page 6, Page 7</t>
+        </is>
+      </c>
       <c r="J105" s="12" t="n">
-        <v>4.38</v>
+        <v>3.46</v>
       </c>
       <c r="K105" s="13" t="inlineStr">
         <is>
@@ -5573,44 +5573,40 @@
       </c>
       <c r="B106" s="17" t="inlineStr">
         <is>
-          <t>Page 9</t>
+          <t>Page 8</t>
         </is>
       </c>
       <c r="C106" s="18" t="inlineStr">
         <is>
-          <t>P4 · MENTAL_SUB  (45 − 12)</t>
+          <t>P3 · PV_SUB  (86 − 56)</t>
         </is>
       </c>
       <c r="D106" s="16" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E106" s="17" t="inlineStr">
         <is>
-          <t>vo_h_order</t>
+          <t>vo_p2_h2</t>
         </is>
       </c>
       <c r="F106" s="19" t="inlineStr">
         <is>
-          <t>संख्याओं में से पहले इकाई में से घटाइए, फिर दहाई में से घटाइए।</t>
+          <t>86 में से 56 घटाने पर, 3 दहाई और 0 इकाई बचती हैं।</t>
         </is>
       </c>
       <c r="G106" s="18" t="inlineStr">
         <is>
-          <t>Hint 1 (1st wrong answer)</t>
+          <t>Hint 2 (2nd wrong answer)</t>
         </is>
       </c>
       <c r="H106" s="18" t="inlineStr">
         <is>
-          <t>the ones digits light on «इकाई», the tens digits on «दहाई»</t>
-        </is>
-      </c>
-      <c r="I106" s="18" t="inlineStr">
-        <is>
-          <t>Page 10</t>
-        </is>
-      </c>
+          <t>the numbers light; the tens and ones left beat on their words</t>
+        </is>
+      </c>
+      <c r="I106" s="18" t="inlineStr"/>
       <c r="J106" s="16" t="n">
-        <v>5.37</v>
+        <v>6.07</v>
       </c>
       <c r="K106" s="17" t="inlineStr">
         <is>
@@ -5624,40 +5620,40 @@
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
-          <t>Page 9</t>
+          <t>Page 8</t>
         </is>
       </c>
       <c r="C107" s="14" t="inlineStr">
         <is>
-          <t>P4 · MENTAL_SUB  (45 − 12)</t>
+          <t>P3 · PV_SUB  (86 − 56)</t>
         </is>
       </c>
       <c r="D107" s="12" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E107" s="13" t="inlineStr">
         <is>
-          <t>vo_p3_h2</t>
+          <t>vo_p2_reveal</t>
         </is>
       </c>
       <c r="F107" s="15" t="inlineStr">
         <is>
-          <t>45 में से 12 घटाने पर, 3 दहाई और 3 इकाई बचती हैं।</t>
+          <t>86 में से 56 घटाने पर 30 बचता है। तो सही संख्या यह है।</t>
         </is>
       </c>
       <c r="G107" s="14" t="inlineStr">
         <is>
-          <t>Hint 2 (2nd wrong answer)</t>
+          <t>Hint 3 (3rd wrong answer)</t>
         </is>
       </c>
       <c r="H107" s="14" t="inlineStr">
         <is>
-          <t>the table comes in with the first number's blocks; the second number is taken away as it is said</t>
+          <t>the right card / the right keys lit (one key at a time), the others off</t>
         </is>
       </c>
       <c r="I107" s="14" t="inlineStr"/>
       <c r="J107" s="12" t="n">
-        <v>5.55</v>
+        <v>5.42</v>
       </c>
       <c r="K107" s="13" t="inlineStr">
         <is>
@@ -5671,40 +5667,40 @@
       </c>
       <c r="B108" s="17" t="inlineStr">
         <is>
-          <t>Page 9</t>
+          <t>Page 8</t>
         </is>
       </c>
       <c r="C108" s="18" t="inlineStr">
         <is>
-          <t>P4 · MENTAL_SUB  (45 − 12)</t>
+          <t>P3 · PV_SUB  (86 − 56)</t>
         </is>
       </c>
       <c r="D108" s="16" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E108" s="17" t="inlineStr">
         <is>
-          <t>vo_p3_reveal</t>
+          <t>vo_p2_correct</t>
         </is>
       </c>
       <c r="F108" s="19" t="inlineStr">
         <is>
-          <t>45 में से 12 घटाने पर 33 बचता है। तो सही संख्या यह है।</t>
+          <t>शाबाश! आपने सही संख्या चुन ली। 86 घटा 56 बराबर 30।</t>
         </is>
       </c>
       <c r="G108" s="18" t="inlineStr">
         <is>
-          <t>Hint 3 (3rd wrong answer)</t>
+          <t>correct answer - first try</t>
         </is>
       </c>
       <c r="H108" s="18" t="inlineStr">
         <is>
-          <t>the right card / the right keys lit (one key at a time), the others off</t>
+          <t>a right answer at the first try: the answer goes into the ?; confetti; the equation's parts light on their words</t>
         </is>
       </c>
       <c r="I108" s="18" t="inlineStr"/>
       <c r="J108" s="16" t="n">
-        <v>5.84</v>
+        <v>7.12</v>
       </c>
       <c r="K108" s="17" t="inlineStr">
         <is>
@@ -5718,44 +5714,44 @@
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
-          <t>Page 9</t>
+          <t>Page 8</t>
         </is>
       </c>
       <c r="C109" s="14" t="inlineStr">
         <is>
-          <t>P4 · MENTAL_SUB  (45 − 12)</t>
+          <t>P3 · PV_SUB  (86 − 56)</t>
         </is>
       </c>
       <c r="D109" s="12" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E109" s="13" t="inlineStr">
         <is>
-          <t>vo_p3_correct</t>
+          <t>vo_p2_correct_plain</t>
         </is>
       </c>
       <c r="F109" s="15" t="inlineStr">
         <is>
-          <t>शाबाश! आपने सही संख्या चुन ली। 45 घटा 12 बराबर 33।</t>
+          <t>आपने सही संख्या चुन ली। 86 घटा 56 बराबर 30।</t>
         </is>
       </c>
       <c r="G109" s="14" t="inlineStr">
         <is>
-          <t>correct answer</t>
+          <t>correct answer - after a wrong try</t>
         </is>
       </c>
       <c r="H109" s="14" t="inlineStr">
         <is>
-          <t>the answer goes into the ?; confetti</t>
+          <t>the same line without «शाबाश!» (cut from it - not recorded separately), after 1-3 wrong tries</t>
         </is>
       </c>
       <c r="I109" s="14" t="inlineStr"/>
       <c r="J109" s="12" t="n">
-        <v>7.59</v>
+        <v>5.87</v>
       </c>
       <c r="K109" s="13" t="inlineStr">
         <is>
-          <t>Recorded (2026-10-27)</t>
+          <t>Cut from vo_p2_correct (tools/make_plain_correct.py)</t>
         </is>
       </c>
     </row>
@@ -5765,12 +5761,12 @@
       </c>
       <c r="B110" s="17" t="inlineStr">
         <is>
-          <t>Page 10</t>
+          <t>Page 9</t>
         </is>
       </c>
       <c r="C110" s="18" t="inlineStr">
         <is>
-          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+          <t>P4 · MENTAL_SUB  (45 − 12)</t>
         </is>
       </c>
       <c r="D110" s="16" t="n">
@@ -5778,12 +5774,12 @@
       </c>
       <c r="E110" s="17" t="inlineStr">
         <is>
-          <t>vo_p67_prompt</t>
+          <t>vo_p3_prompt</t>
         </is>
       </c>
       <c r="F110" s="19" t="inlineStr">
         <is>
-          <t>67 में से 53 घटाइए और सही संख्या चुनिए।</t>
+          <t>45 में से 12 घटाइए और सही संख्या चुनिए।</t>
         </is>
       </c>
       <c r="G110" s="18" t="inlineStr">
@@ -5798,7 +5794,7 @@
       </c>
       <c r="I110" s="18" t="inlineStr"/>
       <c r="J110" s="16" t="n">
-        <v>4.51</v>
+        <v>4.38</v>
       </c>
       <c r="K110" s="17" t="inlineStr">
         <is>
@@ -5812,12 +5808,12 @@
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
-          <t>Page 10</t>
+          <t>Page 9</t>
         </is>
       </c>
       <c r="C111" s="14" t="inlineStr">
         <is>
-          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+          <t>P4 · MENTAL_SUB  (45 − 12)</t>
         </is>
       </c>
       <c r="D111" s="12" t="n">
@@ -5845,7 +5841,7 @@
       </c>
       <c r="I111" s="14" t="inlineStr">
         <is>
-          <t>Page 9</t>
+          <t>Page 10</t>
         </is>
       </c>
       <c r="J111" s="12" t="n">
@@ -5863,12 +5859,12 @@
       </c>
       <c r="B112" s="17" t="inlineStr">
         <is>
-          <t>Page 10</t>
+          <t>Page 9</t>
         </is>
       </c>
       <c r="C112" s="18" t="inlineStr">
         <is>
-          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+          <t>P4 · MENTAL_SUB  (45 − 12)</t>
         </is>
       </c>
       <c r="D112" s="16" t="n">
@@ -5876,12 +5872,12 @@
       </c>
       <c r="E112" s="17" t="inlineStr">
         <is>
-          <t>vo_p67_h2</t>
+          <t>vo_p3_h2</t>
         </is>
       </c>
       <c r="F112" s="19" t="inlineStr">
         <is>
-          <t>67 में से 53 घटाने पर, 1 दहाई और 4 इकाई बचती हैं।</t>
+          <t>45 में से 12 घटाने पर, 3 दहाई और 3 इकाई बचती हैं।</t>
         </is>
       </c>
       <c r="G112" s="18" t="inlineStr">
@@ -5896,7 +5892,7 @@
       </c>
       <c r="I112" s="18" t="inlineStr"/>
       <c r="J112" s="16" t="n">
-        <v>5.7</v>
+        <v>5.55</v>
       </c>
       <c r="K112" s="17" t="inlineStr">
         <is>
@@ -5910,12 +5906,12 @@
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
-          <t>Page 10</t>
+          <t>Page 9</t>
         </is>
       </c>
       <c r="C113" s="14" t="inlineStr">
         <is>
-          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+          <t>P4 · MENTAL_SUB  (45 − 12)</t>
         </is>
       </c>
       <c r="D113" s="12" t="n">
@@ -5923,12 +5919,12 @@
       </c>
       <c r="E113" s="13" t="inlineStr">
         <is>
-          <t>vo_p67_reveal</t>
+          <t>vo_p3_reveal</t>
         </is>
       </c>
       <c r="F113" s="15" t="inlineStr">
         <is>
-          <t>67 में से 53 घटाने पर 14 बचता है। तो सही संख्या यह है।</t>
+          <t>45 में से 12 घटाने पर 33 बचता है। तो सही संख्या यह है।</t>
         </is>
       </c>
       <c r="G113" s="14" t="inlineStr">
@@ -5943,7 +5939,7 @@
       </c>
       <c r="I113" s="14" t="inlineStr"/>
       <c r="J113" s="12" t="n">
-        <v>5.79</v>
+        <v>5.84</v>
       </c>
       <c r="K113" s="13" t="inlineStr">
         <is>
@@ -5957,12 +5953,12 @@
       </c>
       <c r="B114" s="17" t="inlineStr">
         <is>
-          <t>Page 10</t>
+          <t>Page 9</t>
         </is>
       </c>
       <c r="C114" s="18" t="inlineStr">
         <is>
-          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+          <t>P4 · MENTAL_SUB  (45 − 12)</t>
         </is>
       </c>
       <c r="D114" s="16" t="n">
@@ -5970,76 +5966,409 @@
       </c>
       <c r="E114" s="17" t="inlineStr">
         <is>
-          <t>vo_p67_correct</t>
+          <t>vo_p3_correct</t>
         </is>
       </c>
       <c r="F114" s="19" t="inlineStr">
         <is>
-          <t>शाबाश! आपने सही संख्या चुन ली। 67 घटा 53 बराबर 14।</t>
+          <t>शाबाश! आपने सही संख्या चुन ली। 45 घटा 12 बराबर 33।</t>
         </is>
       </c>
       <c r="G114" s="18" t="inlineStr">
         <is>
-          <t>correct answer</t>
+          <t>correct answer - first try</t>
         </is>
       </c>
       <c r="H114" s="18" t="inlineStr">
         <is>
-          <t>the answer goes into the ?; confetti</t>
+          <t>a right answer at the first try: the answer goes into the ?; confetti; the equation's parts light on their words</t>
         </is>
       </c>
       <c r="I114" s="18" t="inlineStr"/>
       <c r="J114" s="16" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="K114" s="17" t="inlineStr">
+        <is>
+          <t>Recorded (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="12" t="n">
+        <v>111</v>
+      </c>
+      <c r="B115" s="13" t="inlineStr">
+        <is>
+          <t>Page 9</t>
+        </is>
+      </c>
+      <c r="C115" s="14" t="inlineStr">
+        <is>
+          <t>P4 · MENTAL_SUB  (45 − 12)</t>
+        </is>
+      </c>
+      <c r="D115" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E115" s="13" t="inlineStr">
+        <is>
+          <t>vo_p3_correct_plain</t>
+        </is>
+      </c>
+      <c r="F115" s="15" t="inlineStr">
+        <is>
+          <t>आपने सही संख्या चुन ली। 45 घटा 12 बराबर 33।</t>
+        </is>
+      </c>
+      <c r="G115" s="14" t="inlineStr">
+        <is>
+          <t>correct answer - after a wrong try</t>
+        </is>
+      </c>
+      <c r="H115" s="14" t="inlineStr">
+        <is>
+          <t>the same line without «शाबाश!» (cut from it - not recorded separately), after 1-3 wrong tries</t>
+        </is>
+      </c>
+      <c r="I115" s="14" t="inlineStr"/>
+      <c r="J115" s="12" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="K115" s="13" t="inlineStr">
+        <is>
+          <t>Cut from vo_p3_correct (tools/make_plain_correct.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="16" t="n">
+        <v>112</v>
+      </c>
+      <c r="B116" s="17" t="inlineStr">
+        <is>
+          <t>Page 10</t>
+        </is>
+      </c>
+      <c r="C116" s="18" t="inlineStr">
+        <is>
+          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+        </is>
+      </c>
+      <c r="D116" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" s="17" t="inlineStr">
+        <is>
+          <t>vo_p67_prompt</t>
+        </is>
+      </c>
+      <c r="F116" s="19" t="inlineStr">
+        <is>
+          <t>67 में से 53 घटाइए और सही संख्या चुनिए।</t>
+        </is>
+      </c>
+      <c r="G116" s="18" t="inlineStr">
+        <is>
+          <t>page instruction</t>
+        </is>
+      </c>
+      <c r="H116" s="18" t="inlineStr">
+        <is>
+          <t>as the page opens (the speaker replays it)</t>
+        </is>
+      </c>
+      <c r="I116" s="18" t="inlineStr"/>
+      <c r="J116" s="16" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="K116" s="17" t="inlineStr">
+        <is>
+          <t>Recorded (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="12" t="n">
+        <v>113</v>
+      </c>
+      <c r="B117" s="13" t="inlineStr">
+        <is>
+          <t>Page 10</t>
+        </is>
+      </c>
+      <c r="C117" s="14" t="inlineStr">
+        <is>
+          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+        </is>
+      </c>
+      <c r="D117" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E117" s="13" t="inlineStr">
+        <is>
+          <t>vo_h_order</t>
+        </is>
+      </c>
+      <c r="F117" s="15" t="inlineStr">
+        <is>
+          <t>संख्याओं में से पहले इकाई में से घटाइए, फिर दहाई में से घटाइए।</t>
+        </is>
+      </c>
+      <c r="G117" s="14" t="inlineStr">
+        <is>
+          <t>Hint 1 (1st wrong answer)</t>
+        </is>
+      </c>
+      <c r="H117" s="14" t="inlineStr">
+        <is>
+          <t>the ones digits light on «इकाई», the tens digits on «दहाई»</t>
+        </is>
+      </c>
+      <c r="I117" s="14" t="inlineStr">
+        <is>
+          <t>Page 9</t>
+        </is>
+      </c>
+      <c r="J117" s="12" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="K117" s="13" t="inlineStr">
+        <is>
+          <t>Recorded (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="16" t="n">
+        <v>114</v>
+      </c>
+      <c r="B118" s="17" t="inlineStr">
+        <is>
+          <t>Page 10</t>
+        </is>
+      </c>
+      <c r="C118" s="18" t="inlineStr">
+        <is>
+          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+        </is>
+      </c>
+      <c r="D118" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E118" s="17" t="inlineStr">
+        <is>
+          <t>vo_p67_h2</t>
+        </is>
+      </c>
+      <c r="F118" s="19" t="inlineStr">
+        <is>
+          <t>67 में से 53 घटाने पर, 1 दहाई और 4 इकाई बचती हैं।</t>
+        </is>
+      </c>
+      <c r="G118" s="18" t="inlineStr">
+        <is>
+          <t>Hint 2 (2nd wrong answer)</t>
+        </is>
+      </c>
+      <c r="H118" s="18" t="inlineStr">
+        <is>
+          <t>the table comes in with the first number's blocks; the second number is taken away as it is said</t>
+        </is>
+      </c>
+      <c r="I118" s="18" t="inlineStr"/>
+      <c r="J118" s="16" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="K118" s="17" t="inlineStr">
+        <is>
+          <t>Recorded (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="12" t="n">
+        <v>115</v>
+      </c>
+      <c r="B119" s="13" t="inlineStr">
+        <is>
+          <t>Page 10</t>
+        </is>
+      </c>
+      <c r="C119" s="14" t="inlineStr">
+        <is>
+          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+        </is>
+      </c>
+      <c r="D119" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E119" s="13" t="inlineStr">
+        <is>
+          <t>vo_p67_reveal</t>
+        </is>
+      </c>
+      <c r="F119" s="15" t="inlineStr">
+        <is>
+          <t>67 में से 53 घटाने पर 14 बचता है। तो सही संख्या यह है।</t>
+        </is>
+      </c>
+      <c r="G119" s="14" t="inlineStr">
+        <is>
+          <t>Hint 3 (3rd wrong answer)</t>
+        </is>
+      </c>
+      <c r="H119" s="14" t="inlineStr">
+        <is>
+          <t>the right card / the right keys lit (one key at a time), the others off</t>
+        </is>
+      </c>
+      <c r="I119" s="14" t="inlineStr"/>
+      <c r="J119" s="12" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="K119" s="13" t="inlineStr">
+        <is>
+          <t>Recorded (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="B120" s="17" t="inlineStr">
+        <is>
+          <t>Page 10</t>
+        </is>
+      </c>
+      <c r="C120" s="18" t="inlineStr">
+        <is>
+          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+        </is>
+      </c>
+      <c r="D120" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E120" s="17" t="inlineStr">
+        <is>
+          <t>vo_p67_correct</t>
+        </is>
+      </c>
+      <c r="F120" s="19" t="inlineStr">
+        <is>
+          <t>शाबाश! आपने सही संख्या चुन ली। 67 घटा 53 बराबर 14।</t>
+        </is>
+      </c>
+      <c r="G120" s="18" t="inlineStr">
+        <is>
+          <t>correct answer - first try</t>
+        </is>
+      </c>
+      <c r="H120" s="18" t="inlineStr">
+        <is>
+          <t>a right answer at the first try: the answer goes into the ?; confetti; the equation's parts light on their words</t>
+        </is>
+      </c>
+      <c r="I120" s="18" t="inlineStr"/>
+      <c r="J120" s="16" t="n">
         <v>6.95</v>
       </c>
-      <c r="K114" s="17" t="inlineStr">
-        <is>
-          <t>Recorded (2026-10-27)</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="20" t="n">
-        <v>111</v>
-      </c>
-      <c r="B115" s="21" t="inlineStr">
+      <c r="K120" s="17" t="inlineStr">
+        <is>
+          <t>Recorded (2026-10-27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="12" t="n">
+        <v>117</v>
+      </c>
+      <c r="B121" s="13" t="inlineStr">
+        <is>
+          <t>Page 10</t>
+        </is>
+      </c>
+      <c r="C121" s="14" t="inlineStr">
+        <is>
+          <t>P5 · MENTAL_SUB  (67 − 53)</t>
+        </is>
+      </c>
+      <c r="D121" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E121" s="13" t="inlineStr">
+        <is>
+          <t>vo_p67_correct_plain</t>
+        </is>
+      </c>
+      <c r="F121" s="15" t="inlineStr">
+        <is>
+          <t>आपने सही संख्या चुन ली। 67 घटा 53 बराबर 14।</t>
+        </is>
+      </c>
+      <c r="G121" s="14" t="inlineStr">
+        <is>
+          <t>correct answer - after a wrong try</t>
+        </is>
+      </c>
+      <c r="H121" s="14" t="inlineStr">
+        <is>
+          <t>the same line without «शाबाश!» (cut from it - not recorded separately), after 1-3 wrong tries</t>
+        </is>
+      </c>
+      <c r="I121" s="14" t="inlineStr"/>
+      <c r="J121" s="12" t="n">
+        <v>5.74</v>
+      </c>
+      <c r="K121" s="13" t="inlineStr">
+        <is>
+          <t>Cut from vo_p67_correct (tools/make_plain_correct.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="20" t="n">
+        <v>118</v>
+      </c>
+      <c r="B122" s="21" t="inlineStr">
         <is>
           <t>Celebration</t>
         </is>
       </c>
-      <c r="C115" s="22" t="inlineStr">
+      <c r="C122" s="22" t="inlineStr">
         <is>
           <t>CEL · CELEBRATION</t>
         </is>
       </c>
-      <c r="D115" s="20" t="n">
+      <c r="D122" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="E115" s="21" t="inlineStr">
+      <c r="E122" s="21" t="inlineStr">
         <is>
           <t>vo_cel</t>
         </is>
       </c>
-      <c r="F115" s="23" t="inlineStr">
+      <c r="F122" s="23" t="inlineStr">
         <is>
           <t>शाबाश! अब आप संख्याएँ घटाना सीख गए हैं।</t>
         </is>
       </c>
-      <c r="G115" s="22" t="inlineStr">
+      <c r="G122" s="22" t="inlineStr">
         <is>
           <t>celebration</t>
         </is>
       </c>
-      <c r="H115" s="22" t="inlineStr">
+      <c r="H122" s="22" t="inlineStr">
         <is>
           <t>the celebration screen: Swiftee jumps on «शाबाश», then says the line lip-synced</t>
         </is>
       </c>
-      <c r="I115" s="22" t="inlineStr"/>
-      <c r="J115" s="20" t="n">
+      <c r="I122" s="22" t="inlineStr"/>
+      <c r="J122" s="20" t="n">
         <v>3.88</v>
       </c>
-      <c r="K115" s="21" t="inlineStr">
+      <c r="K122" s="21" t="inlineStr">
         <is>
           <t>Recorded (2026-10-27)</t>
         </is>
@@ -9115,7 +9444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -9164,7 +9493,7 @@
       </c>
       <c r="B5" s="30" t="inlineStr">
         <is>
-          <t>111 rows, 81 distinct recordings (see 'Recording list'). In the card but not heard in this build (not listed): vo_rm_ones_less, vo_rm_ones_more.</t>
+          <t>118 rows, 81 distinct recordings (see 'Recording list'). In the card but not heard in this build (not listed): vo_rm_ones_less, vo_rm_ones_more.</t>
         </is>
       </c>
     </row>
@@ -9243,34 +9572,46 @@
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
-          <t>Celebration</t>
+          <t>Shabash</t>
         </is>
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>Swiftee's lip-sync on the celebration line is measured from vo_cel.ogg by tools/lessons.py (tools/make_lipsync.py) - re-run it after a new take of vo_cel.</t>
+          <t>A right answer at the FIRST try says the full correct line (with «शाबाश!»); after a wrong try the same line without it - &lt;id&gt;_plain, cut from the recording by tools/make_plain_correct.py (not recorded separately). After a new take of a correct line run it again, then python tools/lessons.py.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>New takes</t>
+          <t>Celebration</t>
         </is>
       </c>
       <c r="B13" s="30" t="inlineStr">
         <is>
-          <t>Put the take in vo_source/recorded/ under its Audio ID (any audio format), then:  python tools/import_vo.py  python tools/lessons.py  and  node tools/gen_asset_sizes.js  (bump the ?v= stamp in index.html so browsers fetch the new audio).</t>
+          <t>Swiftee's lip-sync on the celebration line is measured from vo_cel.ogg by tools/lessons.py (tools/make_lipsync.py) - re-run it after a new take of vo_cel.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
         <is>
+          <t>New takes</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Put the take in vo_source/recorded/ under its Audio ID (any audio format), then:  python tools/import_vo.py  python tools/lessons.py  and  node tools/gen_asset_sizes.js  (bump the ?v= stamp in index.html so browsers fetch the new audio).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
           <t>Regenerate</t>
         </is>
       </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>python tools/gen_vo_manifest.py</t>
         </is>

</xml_diff>